<commit_message>
trust: publish v1.7.4 from smart-trust sitepreview
Take trust/ verbatim from WorldHealthOrganization/smart-trust gh-pages
sitepreview/trust at 7a98019 ("Update sitepreview from v1.7.4 @ bdfc0c3"),
the successful release build that 8844995f97 was meant to publish.

Adds trust/v1.7.4 and comparison-v1.7.3, regenerates the current pages,
package-list.json now lists 1.7.4, and older versions get the usual
"superseded by 1.7.4" release-header update.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0124EVEkZPTcHhiukQZFXZgv
</commit_message>
<xml_diff>
--- a/trust/CodeSystem-Actors.xlsx
+++ b/trust/CodeSystem-Actors.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.7.3</t>
+    <t>1.7.4</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-02T10:11:10+00:00</t>
+    <t>2026-10-12T03:23:53+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>